<commit_message>
feat(phase6/course05): English-only pass, docs truth rewrite, refreshed outputs
- Bilingual strip (nbformat-only) + English agent fixes; zero Arabic in sources and outputs
- Student docs rewritten against OFFICIAL_SPEC facts (hours, official unit titles, single numbered path)
- All notebooks re-executed; parse baseline 0 failures
- Answer-key wording: released by your instructor

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
+++ b/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
@@ -474,10 +474,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D2" t="n">
-        <v>43610.70183540131</v>
+        <v>51441.88693758658</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -498,14 +498,14 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D3" t="n">
-        <v>52433.2962891702</v>
+        <v>32274.97334022658</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -522,14 +522,14 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D4" t="n">
-        <v>65871.40169695686</v>
+        <v>55327.07367630333</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -546,14 +546,14 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D5" t="n">
-        <v>68498.13994245238</v>
+        <v>53883.05560845864</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="D6" t="n">
-        <v>39639.71713924374</v>
+        <v>40650.30729074479</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -594,10 +594,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D7" t="n">
-        <v>42171.93162719346</v>
+        <v>54566.51801959586</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -618,14 +618,14 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="D8" t="n">
-        <v>47556.2125385637</v>
+        <v>47157.23211547599</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="D9" t="n">
-        <v>29129.6189510801</v>
+        <v>27142.38813655752</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -666,14 +666,14 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D10" t="n">
-        <v>59620.6647128093</v>
+        <v>55215.34400981556</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -690,14 +690,14 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="D11" t="n">
-        <v>53488.35558549842</v>
+        <v>27820.06470410521</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -714,14 +714,14 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D12" t="n">
-        <v>38684.7086633722</v>
+        <v>41837.97868262923</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -738,14 +738,14 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D13" t="n">
-        <v>47428.02397843888</v>
+        <v>56911.24976519361</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="D14" t="n">
-        <v>57926.70694848114</v>
+        <v>24481.77896913794</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -786,14 +786,14 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>42264.78411080329</v>
+        <v>67599.34048692118</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -810,14 +810,14 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="D16" t="n">
-        <v>58488.67011243632</v>
+        <v>53899.86491503435</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -834,14 +834,14 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D17" t="n">
-        <v>57041.78768306667</v>
+        <v>34967.91211044697</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -858,14 +858,14 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="D18" t="n">
-        <v>46543.13052467136</v>
+        <v>58906.11010061944</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -882,14 +882,14 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="D19" t="n">
-        <v>25318.51607865423</v>
+        <v>39797.49170877185</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -906,14 +906,14 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="D20" t="n">
-        <v>56919.21861106218</v>
+        <v>48052.83897251657</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -930,10 +930,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D21" t="n">
-        <v>43936.12657109657</v>
+        <v>50413.55055963835</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D22" t="n">
-        <v>38256.24406368241</v>
+        <v>44536.65273905633</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -978,14 +978,14 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D23" t="n">
-        <v>45068.74574912256</v>
+        <v>51604.3899006349</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1002,14 +1002,14 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="D24" t="n">
-        <v>58382.06409465971</v>
+        <v>48917.53313796067</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1026,10 +1026,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="D25" t="n">
-        <v>36028.31514925819</v>
+        <v>53901.19934056902</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1050,14 +1050,14 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="D26" t="n">
-        <v>53211.06209225526</v>
+        <v>52715.34693514708</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1074,14 +1074,14 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D27" t="n">
-        <v>41409.76112369892</v>
+        <v>64172.92242942421</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1098,14 +1098,14 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="D28" t="n">
-        <v>48383.53892505659</v>
+        <v>56494.98518255014</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -1122,14 +1122,14 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="D29" t="n">
-        <v>38842.09039439375</v>
+        <v>63285.21746584714</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -1146,14 +1146,14 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D30" t="n">
-        <v>36787.97008473062</v>
+        <v>47906.49138349226</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1170,10 +1170,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D31" t="n">
-        <v>55725.54683936499</v>
+        <v>48331.18363290506</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1194,14 +1194,14 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D32" t="n">
-        <v>46993.77313027005</v>
+        <v>60595.32421815494</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -1218,14 +1218,14 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D33" t="n">
-        <v>48928.79192061331</v>
+        <v>46071.26317311547</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1242,14 +1242,14 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D34" t="n">
-        <v>17413.88782673988</v>
+        <v>52851.00654145789</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1266,10 +1266,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="D35" t="n">
-        <v>49174.55571784734</v>
+        <v>47533.78456881959</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1290,10 +1290,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D36" t="n">
-        <v>28926.0824343534</v>
+        <v>64570.20948818274</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1314,14 +1314,14 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D37" t="n">
-        <v>44257.10130303896</v>
+        <v>57125.40090092875</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1338,14 +1338,14 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="D38" t="n">
-        <v>48665.60743619078</v>
+        <v>43175.35620727218</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -1362,14 +1362,14 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D39" t="n">
-        <v>34420.82050659293</v>
+        <v>80928.71910314541</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1386,14 +1386,14 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D40" t="n">
-        <v>72066.3945967769</v>
+        <v>58996.79721005342</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -1413,11 +1413,11 @@
         <v>34</v>
       </c>
       <c r="D41" t="n">
-        <v>46332.00469164872</v>
+        <v>65992.30347540962</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1434,14 +1434,14 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="D42" t="n">
-        <v>33869.60721402641</v>
+        <v>24500.09428117785</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -1458,14 +1458,14 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D43" t="n">
-        <v>18699.91143209565</v>
+        <v>41365.95622092973</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -1482,14 +1482,14 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="D44" t="n">
-        <v>48587.04391994402</v>
+        <v>34738.72206484839</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -1506,14 +1506,14 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="D45" t="n">
-        <v>52743.42719405529</v>
+        <v>48176.99411174261</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -1530,10 +1530,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D46" t="n">
-        <v>54757.29635924925</v>
+        <v>62975.05179001259</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1554,10 +1554,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D47" t="n">
-        <v>83582.32280616667</v>
+        <v>63082.2190212952</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1578,14 +1578,14 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D48" t="n">
-        <v>90426.47292622903</v>
+        <v>55865.74371349285</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -1602,14 +1602,14 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D49" t="n">
-        <v>33458.14601254428</v>
+        <v>27483.05961910249</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -1626,14 +1626,14 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="D50" t="n">
-        <v>32041.46274597672</v>
+        <v>62839.83953547929</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -1650,14 +1650,14 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D51" t="n">
-        <v>46318.8371487556</v>
+        <v>45958.20323070223</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -1674,14 +1674,14 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D52" t="n">
-        <v>41251.323595569</v>
+        <v>37751.81464932067</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -1698,10 +1698,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="D53" t="n">
-        <v>44907.97352511045</v>
+        <v>44539.78992961421</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1722,10 +1722,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="D54" t="n">
-        <v>49432.15780874276</v>
+        <v>48003.16387820754</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1746,14 +1746,14 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>74</v>
+        <v>33</v>
       </c>
       <c r="D55" t="n">
-        <v>69732.52410200676</v>
+        <v>47117.23758886647</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -1770,14 +1770,14 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D56" t="n">
-        <v>45614.98154801185</v>
+        <v>47371.67557887234</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -1794,14 +1794,14 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D57" t="n">
-        <v>54648.47410476307</v>
+        <v>69379.62317080906</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -1818,14 +1818,14 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D58" t="n">
-        <v>41229.76005714302</v>
+        <v>76868.17274159777</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -1842,14 +1842,14 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="D59" t="n">
-        <v>38617.70905789319</v>
+        <v>59989.30964138413</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -1866,10 +1866,10 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="D60" t="n">
-        <v>34956.34686184682</v>
+        <v>78817.0135405066</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1890,14 +1890,14 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D61" t="n">
-        <v>63110.62511047053</v>
+        <v>43356.75708305695</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
@@ -1914,14 +1914,14 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D62" t="n">
-        <v>47515.93129972202</v>
+        <v>67254.37125781558</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -1938,14 +1938,14 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D63" t="n">
-        <v>45989.96371295607</v>
+        <v>24918.0370010243</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -1962,14 +1962,14 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="D64" t="n">
-        <v>18988.76630714635</v>
+        <v>47032.87429331854</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
@@ -1986,14 +1986,14 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D65" t="n">
-        <v>68110.38594318964</v>
+        <v>41307.29314431563</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -2010,14 +2010,14 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="D66" t="n">
-        <v>74478.01227269345</v>
+        <v>34586.51394338143</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
@@ -2034,14 +2034,14 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="D67" t="n">
-        <v>44219.46248684295</v>
+        <v>44559.44358248857</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="D68" t="n">
-        <v>40640.11354661808</v>
+        <v>55836.60872370169</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2082,10 +2082,10 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="D69" t="n">
-        <v>69028.9956995003</v>
+        <v>46804.17609171598</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2106,10 +2106,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="D70" t="n">
-        <v>46697.16554013158</v>
+        <v>62717.49074270324</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2130,14 +2130,14 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="D71" t="n">
-        <v>36221.4554323376</v>
+        <v>35271.82565693927</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
@@ -2154,10 +2154,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="D72" t="n">
-        <v>76289.57474945601</v>
+        <v>27724.77666692337</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2178,14 +2178,14 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D73" t="n">
-        <v>51341.706330743</v>
+        <v>31821.62646392227</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -2202,14 +2202,14 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D74" t="n">
-        <v>68832.17569292078</v>
+        <v>57161.25349748486</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -2226,14 +2226,14 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="D75" t="n">
-        <v>36303.4088634776</v>
+        <v>66855.72202615537</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
@@ -2250,14 +2250,14 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="D76" t="n">
-        <v>67951.65293942275</v>
+        <v>38197.81420364216</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -2274,10 +2274,10 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="D77" t="n">
-        <v>63141.25982359784</v>
+        <v>40022.95553394728</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2298,14 +2298,14 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D78" t="n">
-        <v>57652.10090527817</v>
+        <v>34069.60398667793</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
@@ -2322,14 +2322,14 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="D79" t="n">
-        <v>51075.523358577</v>
+        <v>36050.69735739161</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
@@ -2346,10 +2346,10 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D80" t="n">
-        <v>37531.32395948344</v>
+        <v>50956.37913011224</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2370,10 +2370,10 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D81" t="n">
-        <v>57720.94851322562</v>
+        <v>45140.72453276368</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2394,14 +2394,14 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="D82" t="n">
-        <v>46317.43758194576</v>
+        <v>43690.98382901409</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
@@ -2418,14 +2418,14 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="D83" t="n">
-        <v>62790.06141577945</v>
+        <v>55335.65568589298</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
@@ -2442,14 +2442,14 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D84" t="n">
-        <v>63665.13229576965</v>
+        <v>66821.01154119126</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
@@ -2466,14 +2466,14 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="D85" t="n">
-        <v>36374.56798421924</v>
+        <v>41526.47428373132</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
@@ -2490,14 +2490,14 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="D86" t="n">
-        <v>55279.36227607599</v>
+        <v>41310.01727819615</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
@@ -2514,14 +2514,14 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D87" t="n">
-        <v>46908.35148693514</v>
+        <v>52323.60561920475</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
@@ -2538,14 +2538,14 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="D88" t="n">
-        <v>56955.28916720418</v>
+        <v>64440.27149760129</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
@@ -2562,14 +2562,14 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="D89" t="n">
-        <v>69006.98640162079</v>
+        <v>53937.75834073443</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
@@ -2586,14 +2586,14 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D90" t="n">
-        <v>56134.22528998614</v>
+        <v>56819.81529443312</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -2610,10 +2610,10 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="D91" t="n">
-        <v>48497.56888867556</v>
+        <v>63670.66176891895</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2634,14 +2634,14 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="D92" t="n">
-        <v>73460.72856687926</v>
+        <v>40403.50533961868</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
@@ -2658,10 +2658,10 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D93" t="n">
-        <v>30800.79765871239</v>
+        <v>76557.4205570552</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2682,10 +2682,10 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="D94" t="n">
-        <v>82112.42541912582</v>
+        <v>31387.04268608852</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2706,14 +2706,14 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="D95" t="n">
-        <v>70891.61161984793</v>
+        <v>69938.33861999089</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
@@ -2730,14 +2730,14 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D96" t="n">
-        <v>70745.23111122838</v>
+        <v>66802.22219866015</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
@@ -2757,11 +2757,11 @@
         <v>68</v>
       </c>
       <c r="D97" t="n">
-        <v>50735.16097303835</v>
+        <v>53525.95470664815</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
@@ -2778,14 +2778,14 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="D98" t="n">
-        <v>52196.49738872991</v>
+        <v>61712.69108932582</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
@@ -2802,14 +2802,14 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="D99" t="n">
-        <v>48647.59410918901</v>
+        <v>61911.67202295257</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
@@ -2826,10 +2826,10 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D100" t="n">
-        <v>35428.67336017565</v>
+        <v>49616.40700774596</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2850,14 +2850,14 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="D101" t="n">
-        <v>68763.42061738011</v>
+        <v>37049.07402103307</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">

</xml_diff>

<commit_message>
fix(course05/majors): honesty+ordering major findings — computed conclusions, real demos, bridge cells, didactic comments on touched cells
Part of the 13-agent majors wave (all touched notebooks re-executed on their kernels).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
+++ b/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Departments" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,14 +475,14 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D2" t="n">
-        <v>51441.88693758658</v>
+        <v>50256.19363093674</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -498,14 +499,14 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D3" t="n">
-        <v>32274.97334022658</v>
+        <v>50580.49938716307</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -522,10 +523,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="D4" t="n">
-        <v>55327.07367630333</v>
+        <v>34643.09199529465</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -546,14 +547,14 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D5" t="n">
-        <v>53883.05560845864</v>
+        <v>24312.07918587907</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -570,10 +571,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="D6" t="n">
-        <v>40650.30729074479</v>
+        <v>6867.589217373593</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -594,14 +595,14 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D7" t="n">
-        <v>54566.51801959586</v>
+        <v>62104.55931525437</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -618,10 +619,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D8" t="n">
-        <v>47157.23211547599</v>
+        <v>45414.8834754104</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -642,14 +643,14 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D9" t="n">
-        <v>27142.38813655752</v>
+        <v>38699.14219775626</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -666,10 +667,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D10" t="n">
-        <v>55215.34400981556</v>
+        <v>62964.02627578781</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -690,14 +691,14 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" t="n">
-        <v>27820.06470410521</v>
+        <v>65453.52374657642</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -714,14 +715,14 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D12" t="n">
-        <v>41837.97868262923</v>
+        <v>48463.82635962292</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -738,14 +739,14 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D13" t="n">
-        <v>56911.24976519361</v>
+        <v>68375.65560925403</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -762,14 +763,14 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D14" t="n">
-        <v>24481.77896913794</v>
+        <v>33535.77933955527</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -786,14 +787,14 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="D15" t="n">
-        <v>67599.34048692118</v>
+        <v>51059.61515359835</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -810,10 +811,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="D16" t="n">
-        <v>53899.86491503435</v>
+        <v>71048.49756139576</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -834,14 +835,14 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D17" t="n">
-        <v>34967.91211044697</v>
+        <v>58458.49331319515</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -858,14 +859,14 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="D18" t="n">
-        <v>58906.11010061944</v>
+        <v>57717.84721694481</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -882,14 +883,14 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D19" t="n">
-        <v>39797.49170877185</v>
+        <v>70553.6500175898</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -906,14 +907,14 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="D20" t="n">
-        <v>48052.83897251657</v>
+        <v>59440.99030878173</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -930,14 +931,14 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="D21" t="n">
-        <v>50413.55055963835</v>
+        <v>54897.57209055196</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -954,10 +955,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D22" t="n">
-        <v>44536.65273905633</v>
+        <v>45656.75084317962</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -978,14 +979,14 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D23" t="n">
-        <v>51604.3899006349</v>
+        <v>85547.18078532141</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1002,14 +1003,14 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="D24" t="n">
-        <v>48917.53313796067</v>
+        <v>62996.41153470615</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1026,14 +1027,14 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="D25" t="n">
-        <v>53901.19934056902</v>
+        <v>62797.0693955183</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -1050,14 +1051,14 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="D26" t="n">
-        <v>52715.34693514708</v>
+        <v>59027.58911099852</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1074,10 +1075,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D27" t="n">
-        <v>64172.92242942421</v>
+        <v>52039.21906836039</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1098,14 +1099,14 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="D28" t="n">
-        <v>56494.98518255014</v>
+        <v>40529.24222796468</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -1122,10 +1123,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="D29" t="n">
-        <v>63285.21746584714</v>
+        <v>44430.10005804124</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1146,14 +1147,14 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D30" t="n">
-        <v>47906.49138349226</v>
+        <v>56477.87095227242</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1170,14 +1171,14 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="D31" t="n">
-        <v>48331.18363290506</v>
+        <v>41290.19098125486</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1194,14 +1195,14 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="D32" t="n">
-        <v>60595.32421815494</v>
+        <v>65048.19385017278</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -1218,10 +1219,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="D33" t="n">
-        <v>46071.26317311547</v>
+        <v>64671.77990184991</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1242,14 +1243,14 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D34" t="n">
-        <v>52851.00654145789</v>
+        <v>44694.21955223565</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1266,14 +1267,14 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D35" t="n">
-        <v>47533.78456881959</v>
+        <v>65648.69717967423</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -1290,10 +1291,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="D36" t="n">
-        <v>64570.20948818274</v>
+        <v>62182.11987095779</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1314,14 +1315,14 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D37" t="n">
-        <v>57125.40090092875</v>
+        <v>68120.49640273306</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1338,10 +1339,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D38" t="n">
-        <v>43175.35620727218</v>
+        <v>55595.14096856588</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1362,14 +1363,14 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D39" t="n">
-        <v>80928.71910314541</v>
+        <v>37272.22335067701</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1386,14 +1387,14 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="D40" t="n">
-        <v>58996.79721005342</v>
+        <v>55607.63226731973</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -1410,10 +1411,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="D41" t="n">
-        <v>65992.30347540962</v>
+        <v>58611.18079231313</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1434,14 +1435,14 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D42" t="n">
-        <v>24500.09428117785</v>
+        <v>63910.00502615862</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -1458,10 +1459,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D43" t="n">
-        <v>41365.95622092973</v>
+        <v>24559.93629114584</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1482,14 +1483,14 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="D44" t="n">
-        <v>34738.72206484839</v>
+        <v>68579.96807455293</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -1506,14 +1507,14 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="D45" t="n">
-        <v>48176.99411174261</v>
+        <v>52889.78006292566</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -1530,14 +1531,14 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D46" t="n">
-        <v>62975.05179001259</v>
+        <v>74713.39819882849</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -1554,10 +1555,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D47" t="n">
-        <v>63082.2190212952</v>
+        <v>33615.62477401169</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1578,10 +1579,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D48" t="n">
-        <v>55865.74371349285</v>
+        <v>50462.2845734474</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1602,10 +1603,10 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="D49" t="n">
-        <v>27483.05961910249</v>
+        <v>33508.315317209</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1626,14 +1627,14 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D50" t="n">
-        <v>62839.83953547929</v>
+        <v>78360.17770655997</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -1650,14 +1651,14 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D51" t="n">
-        <v>45958.20323070223</v>
+        <v>24367.13395418666</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -1674,14 +1675,14 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="D52" t="n">
-        <v>37751.81464932067</v>
+        <v>13670.71657079629</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -1698,14 +1699,14 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D53" t="n">
-        <v>44539.78992961421</v>
+        <v>42881.7249942844</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
@@ -1722,14 +1723,14 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="D54" t="n">
-        <v>48003.16387820754</v>
+        <v>55214.23347126509</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
@@ -1746,14 +1747,14 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="D55" t="n">
-        <v>47117.23758886647</v>
+        <v>24913.58359956947</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -1770,14 +1771,14 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="D56" t="n">
-        <v>47371.67557887234</v>
+        <v>93799.55312704112</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -1794,14 +1795,14 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D57" t="n">
-        <v>69379.62317080906</v>
+        <v>63093.61149063162</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -1818,14 +1819,14 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="D58" t="n">
-        <v>76868.17274159777</v>
+        <v>46329.41836815349</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -1842,14 +1843,14 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D59" t="n">
-        <v>59989.30964138413</v>
+        <v>43415.02517522644</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -1866,14 +1867,14 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="D60" t="n">
-        <v>78817.0135405066</v>
+        <v>43241.04112211792</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
@@ -1890,14 +1891,14 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="D61" t="n">
-        <v>43356.75708305695</v>
+        <v>63761.30878031984</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
@@ -1914,14 +1915,14 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D62" t="n">
-        <v>67254.37125781558</v>
+        <v>49851.29313785893</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -1938,14 +1939,14 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="D63" t="n">
-        <v>24918.0370010243</v>
+        <v>61751.68752015456</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -1962,14 +1963,14 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="D64" t="n">
-        <v>47032.87429331854</v>
+        <v>19988.66066399444</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
@@ -1986,10 +1987,10 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="D65" t="n">
-        <v>41307.29314431563</v>
+        <v>57996.0906309112</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2010,14 +2011,14 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="D66" t="n">
-        <v>34586.51394338143</v>
+        <v>64287.95401721614</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
@@ -2034,14 +2035,14 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D67" t="n">
-        <v>44559.44358248857</v>
+        <v>57692.58647429774</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -2058,14 +2059,14 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D68" t="n">
-        <v>55836.60872370169</v>
+        <v>54883.82800958731</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
@@ -2082,14 +2083,14 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="D69" t="n">
-        <v>46804.17609171598</v>
+        <v>41850.63050739581</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
@@ -2106,10 +2107,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="D70" t="n">
-        <v>62717.49074270324</v>
+        <v>56657.6736851145</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2130,14 +2131,14 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="D71" t="n">
-        <v>35271.82565693927</v>
+        <v>73864.91192708215</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
@@ -2154,14 +2155,14 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="D72" t="n">
-        <v>27724.77666692337</v>
+        <v>46102.30628559215</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
@@ -2178,14 +2179,14 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="D73" t="n">
-        <v>31821.62646392227</v>
+        <v>57991.10988060255</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -2202,14 +2203,14 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D74" t="n">
-        <v>57161.25349748486</v>
+        <v>50244.37794746801</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -2226,14 +2227,14 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="D75" t="n">
-        <v>66855.72202615537</v>
+        <v>45617.32092520866</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
@@ -2250,14 +2251,14 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="D76" t="n">
-        <v>38197.81420364216</v>
+        <v>62116.20679300049</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -2274,14 +2275,14 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D77" t="n">
-        <v>40022.95553394728</v>
+        <v>49397.54771443936</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
@@ -2298,14 +2299,14 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="D78" t="n">
-        <v>34069.60398667793</v>
+        <v>73111.65711463371</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
@@ -2322,14 +2323,14 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="D79" t="n">
-        <v>36050.69735739161</v>
+        <v>55796.08859070885</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
@@ -2346,14 +2347,14 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="D80" t="n">
-        <v>50956.37913011224</v>
+        <v>83245.95004334343</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
@@ -2370,14 +2371,14 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="D81" t="n">
-        <v>45140.72453276368</v>
+        <v>58341.30871540195</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
@@ -2394,14 +2395,14 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D82" t="n">
-        <v>43690.98382901409</v>
+        <v>33781.50357195373</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
@@ -2418,14 +2419,14 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="D83" t="n">
-        <v>55335.65568589298</v>
+        <v>21591.18134210139</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
@@ -2442,10 +2443,10 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D84" t="n">
-        <v>66821.01154119126</v>
+        <v>52888.99100554134</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2466,10 +2467,10 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D85" t="n">
-        <v>41526.47428373132</v>
+        <v>49899.59185407408</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2490,14 +2491,14 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="D86" t="n">
-        <v>41310.01727819615</v>
+        <v>58189.82684545925</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
@@ -2514,14 +2515,14 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="D87" t="n">
-        <v>52323.60561920475</v>
+        <v>43060.42583492932</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
@@ -2538,10 +2539,10 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D88" t="n">
-        <v>64440.27149760129</v>
+        <v>40251.11127908823</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2562,14 +2563,14 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="D89" t="n">
-        <v>53937.75834073443</v>
+        <v>62905.74924616493</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
@@ -2586,14 +2587,14 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="D90" t="n">
-        <v>56819.81529443312</v>
+        <v>76304.44565447468</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -2610,14 +2611,14 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D91" t="n">
-        <v>63670.66176891895</v>
+        <v>44477.40448003981</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
@@ -2634,14 +2635,14 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="D92" t="n">
-        <v>40403.50533961868</v>
+        <v>48343.54008506146</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
@@ -2658,14 +2659,14 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D93" t="n">
-        <v>76557.4205570552</v>
+        <v>51084.11646695972</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F93" s="2" t="n">
@@ -2682,14 +2683,14 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D94" t="n">
-        <v>31387.04268608852</v>
+        <v>55527.98645204119</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
@@ -2706,14 +2707,14 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="D95" t="n">
-        <v>69938.33861999089</v>
+        <v>73808.58345902609</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
@@ -2730,14 +2731,14 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="D96" t="n">
-        <v>66802.22219866015</v>
+        <v>35740.5850512209</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
@@ -2754,14 +2755,14 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="D97" t="n">
-        <v>53525.95470664815</v>
+        <v>67044.22790367773</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
@@ -2778,10 +2779,10 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D98" t="n">
-        <v>61712.69108932582</v>
+        <v>72063.43984961871</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2802,14 +2803,14 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D99" t="n">
-        <v>61911.67202295257</v>
+        <v>38149.17638236816</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
@@ -2826,10 +2827,10 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D100" t="n">
-        <v>49616.40700774596</v>
+        <v>51297.338391632</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2850,18 +2851,88 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="D101" t="n">
-        <v>37049.07402103307</v>
+        <v>35811.45408789709</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
         <v>43930</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dept_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dept_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>budget_k</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(course05/polish): didactic comments in every substantive code cell + verified References (seminal + recent papers) in every lesson
Comment-density gate: zero bare cells. Citations fetch-verified (post-2020 and off-anchor entries); classics cited without links where publishers block fetching. All touched notebooks re-executed on their kernels.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
+++ b/Course 05/unit2-cleaning/examples/unit2-cleaning/examples/sample_data.xlsx
@@ -475,14 +475,14 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D2" t="n">
-        <v>50256.19363093674</v>
+        <v>72482.93259557607</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -499,14 +499,14 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="D3" t="n">
-        <v>50580.49938716307</v>
+        <v>84641.07082561411</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -523,14 +523,14 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="D4" t="n">
-        <v>34643.09199529465</v>
+        <v>43366.06904224229</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -547,14 +547,14 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="D5" t="n">
-        <v>24312.07918587907</v>
+        <v>29265.87817950248</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -571,14 +571,14 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>6867.589217373593</v>
+        <v>33476.77383653756</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -595,14 +595,14 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D7" t="n">
-        <v>62104.55931525437</v>
+        <v>55071.45663758033</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="D8" t="n">
-        <v>45414.8834754104</v>
+        <v>24115.26192157633</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -643,14 +643,14 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D9" t="n">
-        <v>38699.14219775626</v>
+        <v>30356.04359882229</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D10" t="n">
-        <v>62964.02627578781</v>
+        <v>51875.19137069861</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -691,14 +691,14 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="D11" t="n">
-        <v>65453.52374657642</v>
+        <v>69410.37102719663</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -715,14 +715,14 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D12" t="n">
-        <v>48463.82635962292</v>
+        <v>64955.317123197</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" t="n">
-        <v>68375.65560925403</v>
+        <v>36923.02824923709</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -763,14 +763,14 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D14" t="n">
-        <v>33535.77933955527</v>
+        <v>41576.64786205359</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -787,10 +787,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="D15" t="n">
-        <v>51059.61515359835</v>
+        <v>53381.67872027891</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -811,14 +811,14 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D16" t="n">
-        <v>71048.49756139576</v>
+        <v>46622.90638362621</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -835,14 +835,14 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D17" t="n">
-        <v>58458.49331319515</v>
+        <v>72384.59992589659</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -859,10 +859,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D18" t="n">
-        <v>57717.84721694481</v>
+        <v>59036.94060577649</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -883,14 +883,14 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D19" t="n">
-        <v>70553.6500175898</v>
+        <v>59355.08046981548</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -907,14 +907,14 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="D20" t="n">
-        <v>59440.99030878173</v>
+        <v>50471.63705983343</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -931,10 +931,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="D21" t="n">
-        <v>54897.57209055196</v>
+        <v>44015.20456566104</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -955,14 +955,14 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="D22" t="n">
-        <v>45656.75084317962</v>
+        <v>47179.3408733183</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -979,14 +979,14 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="D23" t="n">
-        <v>85547.18078532141</v>
+        <v>53017.61786217989</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1003,14 +1003,14 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>62996.41153470615</v>
+        <v>20923.27726473957</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1027,10 +1027,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D25" t="n">
-        <v>62797.0693955183</v>
+        <v>54483.74546966386</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1051,14 +1051,14 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="D26" t="n">
-        <v>59027.58911099852</v>
+        <v>50740.62368139847</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1075,14 +1075,14 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="D27" t="n">
-        <v>52039.21906836039</v>
+        <v>61962.12147625707</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1099,14 +1099,14 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D28" t="n">
-        <v>40529.24222796468</v>
+        <v>52989.31216243831</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -1123,14 +1123,14 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="D29" t="n">
-        <v>44430.10005804124</v>
+        <v>46673.55860647591</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -1147,14 +1147,14 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="D30" t="n">
-        <v>56477.87095227242</v>
+        <v>58000.04412580726</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1171,14 +1171,14 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="D31" t="n">
-        <v>41290.19098125486</v>
+        <v>63210.69300527598</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="D32" t="n">
-        <v>65048.19385017278</v>
+        <v>71540.26024168955</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1219,14 +1219,14 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="D33" t="n">
-        <v>64671.77990184991</v>
+        <v>46865.75306593465</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1243,10 +1243,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="D34" t="n">
-        <v>44694.21955223565</v>
+        <v>51668.70250853756</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1267,14 +1267,14 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D35" t="n">
-        <v>65648.69717967423</v>
+        <v>54183.63045820544</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -1291,14 +1291,14 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="D36" t="n">
-        <v>62182.11987095779</v>
+        <v>39989.17504170147</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1315,14 +1315,14 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="D37" t="n">
-        <v>68120.49640273306</v>
+        <v>34088.36318872555</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1339,14 +1339,14 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D38" t="n">
-        <v>55595.14096856588</v>
+        <v>50324.5738338862</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -1363,14 +1363,14 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="D39" t="n">
-        <v>37272.22335067701</v>
+        <v>34463.81972428848</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1387,14 +1387,14 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="D40" t="n">
-        <v>55607.63226731973</v>
+        <v>70346.79188557882</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -1411,10 +1411,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D41" t="n">
-        <v>58611.18079231313</v>
+        <v>62754.71615219959</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1435,10 +1435,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D42" t="n">
-        <v>63910.00502615862</v>
+        <v>47363.82865489121</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1459,14 +1459,14 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D43" t="n">
-        <v>24559.93629114584</v>
+        <v>43563.56615508557</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -1483,14 +1483,14 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D44" t="n">
-        <v>68579.96807455293</v>
+        <v>63800.67404637535</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -1507,14 +1507,14 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D45" t="n">
-        <v>52889.78006292566</v>
+        <v>26393.1946612443</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -1531,14 +1531,14 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D46" t="n">
-        <v>74713.39819882849</v>
+        <v>49234.84004097966</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -1555,14 +1555,14 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="D47" t="n">
-        <v>33615.62477401169</v>
+        <v>43705.60516505804</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -1582,7 +1582,7 @@
         <v>45</v>
       </c>
       <c r="D48" t="n">
-        <v>50462.2845734474</v>
+        <v>52549.86804291635</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1603,14 +1603,14 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D49" t="n">
-        <v>33508.315317209</v>
+        <v>31628.19650175522</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -1627,14 +1627,14 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>64</v>
+        <v>19</v>
       </c>
       <c r="D50" t="n">
-        <v>78360.17770655997</v>
+        <v>28389.9803065272</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -1651,14 +1651,14 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D51" t="n">
-        <v>24367.13395418666</v>
+        <v>28704.22142379697</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -1675,14 +1675,14 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="D52" t="n">
-        <v>13670.71657079629</v>
+        <v>57917.63503709918</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D53" t="n">
-        <v>42881.7249942844</v>
+        <v>40198.17994307771</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1723,14 +1723,14 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D54" t="n">
-        <v>55214.23347126509</v>
+        <v>39454.19643292623</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
@@ -1747,14 +1747,14 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="D55" t="n">
-        <v>24913.58359956947</v>
+        <v>32816.21087856179</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -1771,14 +1771,14 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D56" t="n">
-        <v>93799.55312704112</v>
+        <v>46499.66272673524</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -1795,10 +1795,10 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D57" t="n">
-        <v>63093.61149063162</v>
+        <v>41398.31086485468</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1819,14 +1819,14 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="D58" t="n">
-        <v>46329.41836815349</v>
+        <v>56153.29486723421</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -1843,14 +1843,14 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="D59" t="n">
-        <v>43415.02517522644</v>
+        <v>79542.63115644331</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -1867,14 +1867,14 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="D60" t="n">
-        <v>43241.04112211792</v>
+        <v>61097.60414457617</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
@@ -1894,7 +1894,7 @@
         <v>61</v>
       </c>
       <c r="D61" t="n">
-        <v>63761.30878031984</v>
+        <v>71744.60883597471</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1915,14 +1915,14 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="D62" t="n">
-        <v>49851.29313785893</v>
+        <v>39963.79199859873</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -1939,14 +1939,14 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="D63" t="n">
-        <v>61751.68752015456</v>
+        <v>44682.45189062759</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -1963,14 +1963,14 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D64" t="n">
-        <v>19988.66066399444</v>
+        <v>38005.23458894687</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
@@ -1987,14 +1987,14 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D65" t="n">
-        <v>57996.0906309112</v>
+        <v>62057.49451323243</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -2011,14 +2011,14 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D66" t="n">
-        <v>64287.95401721614</v>
+        <v>58893.48712720442</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
@@ -2035,14 +2035,14 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="D67" t="n">
-        <v>57692.58647429774</v>
+        <v>44174.24068065577</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
@@ -2062,11 +2062,11 @@
         <v>71</v>
       </c>
       <c r="D68" t="n">
-        <v>54883.82800958731</v>
+        <v>77989.11441076186</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
@@ -2083,14 +2083,14 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D69" t="n">
-        <v>41850.63050739581</v>
+        <v>35873.45178370208</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
@@ -2107,14 +2107,14 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="D70" t="n">
-        <v>56657.6736851145</v>
+        <v>62644.44998379859</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
@@ -2131,14 +2131,14 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="D71" t="n">
-        <v>73864.91192708215</v>
+        <v>26603.42779478489</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
@@ -2155,14 +2155,14 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="D72" t="n">
-        <v>46102.30628559215</v>
+        <v>27447.41739973784</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
@@ -2179,14 +2179,14 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="D73" t="n">
-        <v>57991.10988060255</v>
+        <v>52032.48917216058</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -2203,14 +2203,14 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="D74" t="n">
-        <v>50244.37794746801</v>
+        <v>46938.10788704598</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -2227,14 +2227,14 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="D75" t="n">
-        <v>45617.32092520866</v>
+        <v>63342.3032068801</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
@@ -2251,14 +2251,14 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D76" t="n">
-        <v>62116.20679300049</v>
+        <v>54414.08859677181</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -2275,10 +2275,10 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D77" t="n">
-        <v>49397.54771443936</v>
+        <v>66981.15277899572</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2299,10 +2299,10 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="D78" t="n">
-        <v>73111.65711463371</v>
+        <v>31618.96149609431</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2323,14 +2323,14 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="D79" t="n">
-        <v>55796.08859070885</v>
+        <v>57607.17850704381</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
@@ -2347,10 +2347,10 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="D80" t="n">
-        <v>83245.95004334343</v>
+        <v>32368.69436532991</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2371,14 +2371,14 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D81" t="n">
-        <v>58341.30871540195</v>
+        <v>20020.48581643611</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
@@ -2395,10 +2395,10 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="D82" t="n">
-        <v>33781.50357195373</v>
+        <v>72702.88197096827</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2419,14 +2419,14 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D83" t="n">
-        <v>21591.18134210139</v>
+        <v>38483.62864972488</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
@@ -2443,10 +2443,10 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D84" t="n">
-        <v>52888.99100554134</v>
+        <v>43573.1703943194</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2467,14 +2467,14 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D85" t="n">
-        <v>49899.59185407408</v>
+        <v>60350.08012923896</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
@@ -2491,14 +2491,14 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="D86" t="n">
-        <v>58189.82684545925</v>
+        <v>61889.12840632362</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
@@ -2515,14 +2515,14 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D87" t="n">
-        <v>43060.42583492932</v>
+        <v>52349.34446543391</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
@@ -2539,14 +2539,14 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D88" t="n">
-        <v>40251.11127908823</v>
+        <v>58398.96790777916</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
@@ -2563,10 +2563,10 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="D89" t="n">
-        <v>62905.74924616493</v>
+        <v>58509.4695288834</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2587,14 +2587,14 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D90" t="n">
-        <v>76304.44565447468</v>
+        <v>42646.28584418391</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -2611,14 +2611,14 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D91" t="n">
-        <v>44477.40448003981</v>
+        <v>42129.94543679679</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
@@ -2635,14 +2635,14 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D92" t="n">
-        <v>48343.54008506146</v>
+        <v>64822.97900624468</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
@@ -2659,14 +2659,14 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D93" t="n">
-        <v>51084.11646695972</v>
+        <v>63161.84265204908</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F93" s="2" t="n">
@@ -2683,14 +2683,14 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="D94" t="n">
-        <v>55527.98645204119</v>
+        <v>30447.22343822998</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
@@ -2707,14 +2707,14 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="D95" t="n">
-        <v>73808.58345902609</v>
+        <v>22947.97485101244</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
@@ -2731,10 +2731,10 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D96" t="n">
-        <v>35740.5850512209</v>
+        <v>39896.98006459441</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2755,14 +2755,14 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D97" t="n">
-        <v>67044.22790367773</v>
+        <v>52630.42188377498</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
@@ -2779,14 +2779,14 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="D98" t="n">
-        <v>72063.43984961871</v>
+        <v>40310.48444940572</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
@@ -2803,10 +2803,10 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="D99" t="n">
-        <v>38149.17638236816</v>
+        <v>70033.8629462199</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2827,14 +2827,14 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="D100" t="n">
-        <v>51297.338391632</v>
+        <v>30527.14713673857</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
@@ -2851,14 +2851,14 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="D101" t="n">
-        <v>35811.45408789709</v>
+        <v>29322.44264802228</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">

</xml_diff>